<commit_message>
- Modifiqué visualizacion_datos - Modifiqué extras para que se guarden
</commit_message>
<xml_diff>
--- a/Carga_Diego2.xlsx
+++ b/Carga_Diego2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="ON" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="265">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -353,9 +353,6 @@
     <t xml:space="preserve">Silver Endeavour</t>
   </si>
   <si>
-    <t xml:space="preserve">32-12-2024</t>
-  </si>
-  <si>
     <t xml:space="preserve">Puerto Williams</t>
   </si>
   <si>
@@ -522,6 +519,9 @@
   </si>
   <si>
     <t xml:space="preserve">Cabo de Hornos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NO</t>
   </si>
   <si>
     <t xml:space="preserve">SCHMIDT</t>
@@ -838,7 +838,7 @@
     <numFmt numFmtId="173" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="174" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -877,7 +877,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
       <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -886,12 +885,6 @@
     <font>
       <sz val="8"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -1017,7 +1010,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="75">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1182,95 +1175,123 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1278,47 +1299,15 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1837,7 +1826,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" s="45" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="37" t="s">
         <v>106</v>
       </c>
@@ -1848,59 +1837,59 @@
         <v>108</v>
       </c>
       <c r="D2" s="39"/>
-      <c r="E2" s="39" t="s">
+      <c r="E2" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F2" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G2" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="F2" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G2" s="38" t="s">
+      <c r="H2" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="H2" s="38" t="s">
+      <c r="I2" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="38" t="s">
+      <c r="J2" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="K2" s="40" t="s">
         <v>112</v>
       </c>
-      <c r="J2" s="38" t="s">
-        <v>112</v>
-      </c>
-      <c r="K2" s="40" t="s">
+      <c r="L2" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="L2" s="40" t="s">
+      <c r="M2" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="M2" s="41" t="s">
+      <c r="N2" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="N2" s="40" t="s">
+      <c r="O2" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="O2" s="40" t="s">
+      <c r="P2" s="38" t="s">
         <v>117</v>
       </c>
-      <c r="P2" s="38" t="s">
+      <c r="Q2" s="41" t="n">
+        <v>32251</v>
+      </c>
+      <c r="R2" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="Q2" s="42" t="n">
-        <v>32251</v>
-      </c>
-      <c r="R2" s="40" t="s">
+      <c r="S2" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="T2" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="S2" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="T2" s="40" t="s">
+      <c r="U2" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="U2" s="38" t="s">
+      <c r="V2" s="40" t="s">
         <v>121</v>
-      </c>
-      <c r="V2" s="40" t="s">
-        <v>122</v>
       </c>
       <c r="W2" s="39" t="n">
         <v>45608</v>
@@ -1909,74 +1898,74 @@
         <v>0.288194444444444</v>
       </c>
       <c r="Y2" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Z2" s="39" t="n">
         <v>45609</v>
       </c>
       <c r="AA2" s="39" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB2" s="38" t="s">
         <v>124</v>
-      </c>
-      <c r="AB2" s="38" t="s">
-        <v>125</v>
       </c>
       <c r="AC2" s="39" t="n">
         <v>45609</v>
       </c>
       <c r="AD2" s="39" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AE2" s="38"/>
       <c r="AF2" s="38"/>
       <c r="AG2" s="38"/>
       <c r="AH2" s="40" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AI2" s="39" t="n">
         <v>45609</v>
       </c>
-      <c r="AJ2" s="43" t="s">
+      <c r="AJ2" s="42" t="s">
+        <v>126</v>
+      </c>
+      <c r="AK2" s="38" t="s">
         <v>127</v>
-      </c>
-      <c r="AK2" s="38" t="s">
-        <v>128</v>
       </c>
       <c r="AL2" s="39" t="n">
         <v>45610</v>
       </c>
-      <c r="AM2" s="44" t="s">
+      <c r="AM2" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="AN2" s="38" t="s">
         <v>129</v>
       </c>
-      <c r="AN2" s="38" t="s">
+      <c r="AO2" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="AP2" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="AO2" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="AP2" s="39" t="s">
+      <c r="AQ2" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="AQ2" s="38" t="s">
+      <c r="AR2" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="AR2" s="38" t="s">
+      <c r="AS2" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="AS2" s="38" t="s">
+      <c r="AT2" s="38" t="s">
         <v>134</v>
-      </c>
-      <c r="AT2" s="38" t="s">
-        <v>135</v>
       </c>
       <c r="AU2" s="38"/>
       <c r="AV2" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW2" s="38" t="n">
         <v>3</v>
       </c>
       <c r="AX2" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AY2" s="39" t="n">
         <v>45610</v>
@@ -1985,10 +1974,10 @@
         <v>45612</v>
       </c>
       <c r="BA2" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="BB2" s="38" t="s">
         <v>138</v>
-      </c>
-      <c r="BB2" s="38" t="s">
-        <v>139</v>
       </c>
       <c r="BC2" s="38"/>
       <c r="BD2" s="39"/>
@@ -2001,57 +1990,57 @@
       <c r="BK2" s="38"/>
       <c r="BL2" s="38"/>
       <c r="BM2" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN2" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BN2" s="38" t="s">
+      <c r="BO2" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP2" s="38" t="s">
         <v>141</v>
-      </c>
-      <c r="BO2" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="BP2" s="38" t="s">
-        <v>142</v>
       </c>
       <c r="BQ2" s="39" t="n">
         <v>45610</v>
       </c>
-      <c r="BR2" s="43" t="n">
+      <c r="BR2" s="42" t="n">
         <v>0.329166666666667</v>
       </c>
       <c r="BS2" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT2" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU2" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV2" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BT2" s="38" t="s">
+      <c r="BW2" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BX2" s="42" t="n">
+        <v>0.145833333333333</v>
+      </c>
+      <c r="BY2" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="BU2" s="38" t="s">
+      <c r="BZ2" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="BV2" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW2" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BX2" s="43" t="n">
-        <v>0.145833333333333</v>
-      </c>
-      <c r="BY2" s="38" t="s">
+      <c r="CA2" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="CB2" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="BZ2" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="CA2" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="CB2" s="38" t="s">
-        <v>144</v>
-      </c>
       <c r="CC2" s="39" t="n">
         <v>45612</v>
       </c>
-      <c r="CD2" s="43" t="n">
+      <c r="CD2" s="42" t="n">
         <v>0.28125</v>
       </c>
       <c r="CE2" s="39"/>
@@ -2062,35 +2051,41 @@
       <c r="CJ2" s="39"/>
       <c r="CK2" s="38"/>
       <c r="CL2" s="38" t="s">
-        <v>145</v>
-      </c>
-      <c r="CM2" s="42" t="n">
+        <v>144</v>
+      </c>
+      <c r="CM2" s="41" t="n">
         <v>42688</v>
       </c>
-      <c r="CN2" s="42" t="n">
+      <c r="CN2" s="41" t="n">
         <v>45611</v>
       </c>
       <c r="CO2" s="38"/>
       <c r="CP2" s="38" t="s">
-        <v>146</v>
-      </c>
-      <c r="CQ2" s="42" t="n">
+        <v>145</v>
+      </c>
+      <c r="CQ2" s="41" t="n">
         <v>45610</v>
       </c>
-      <c r="CR2" s="42" t="n">
+      <c r="CR2" s="41" t="n">
         <v>45611</v>
       </c>
-      <c r="CS2" s="41"/>
+      <c r="CS2" s="37"/>
       <c r="CT2" s="38"/>
       <c r="CU2" s="39"/>
       <c r="CV2" s="38"/>
+      <c r="CX2" s="44" t="s">
+        <v>106</v>
+      </c>
+      <c r="CZ2" s="44" t="s">
+        <v>106</v>
+      </c>
     </row>
-    <row r="3" s="45" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="41" t="s">
+    <row r="3" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="37" t="s">
         <v>106</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C3" s="38" t="s">
         <v>108</v>
@@ -2103,128 +2098,128 @@
         <v>45612</v>
       </c>
       <c r="G3" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="H3" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="H3" s="38" t="s">
+      <c r="I3" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="38" t="s">
-        <v>112</v>
-      </c>
       <c r="J3" s="38" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K3" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="L3" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="L3" s="40" t="s">
+      <c r="M3" s="37" t="s">
         <v>149</v>
       </c>
-      <c r="M3" s="41" t="s">
+      <c r="N3" s="40" t="s">
         <v>150</v>
       </c>
-      <c r="N3" s="40" t="s">
+      <c r="O3" s="40" t="s">
         <v>151</v>
       </c>
-      <c r="O3" s="40" t="s">
+      <c r="P3" s="38" t="s">
         <v>152</v>
       </c>
-      <c r="P3" s="38" t="s">
+      <c r="Q3" s="41" t="n">
+        <v>21685</v>
+      </c>
+      <c r="R3" s="40" t="s">
         <v>153</v>
       </c>
-      <c r="Q3" s="42" t="n">
-        <v>21685</v>
-      </c>
-      <c r="R3" s="40" t="s">
+      <c r="S3" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="T3" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="U3" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="V3" s="40" t="s">
         <v>154</v>
-      </c>
-      <c r="S3" s="40" t="s">
-        <v>120</v>
-      </c>
-      <c r="T3" s="40" t="s">
-        <v>120</v>
-      </c>
-      <c r="U3" s="38" t="s">
-        <v>121</v>
-      </c>
-      <c r="V3" s="40" t="s">
-        <v>155</v>
       </c>
       <c r="W3" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="X3" s="39" t="s">
+        <v>155</v>
+      </c>
+      <c r="Y3" s="38" t="s">
         <v>156</v>
-      </c>
-      <c r="Y3" s="38" t="s">
-        <v>157</v>
       </c>
       <c r="Z3" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="AA3" s="39" t="s">
+        <v>157</v>
+      </c>
+      <c r="AB3" s="38" t="s">
         <v>158</v>
-      </c>
-      <c r="AB3" s="38" t="s">
-        <v>159</v>
       </c>
       <c r="AC3" s="39" t="n">
         <v>45611</v>
       </c>
       <c r="AD3" s="39" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AE3" s="38"/>
       <c r="AF3" s="38"/>
       <c r="AG3" s="38"/>
       <c r="AH3" s="40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AI3" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AJ3" s="43" t="s">
+      <c r="AJ3" s="42" t="s">
+        <v>160</v>
+      </c>
+      <c r="AK3" s="45" t="s">
         <v>161</v>
-      </c>
-      <c r="AK3" s="46" t="s">
-        <v>162</v>
       </c>
       <c r="AL3" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AM3" s="47" t="s">
-        <v>163</v>
-      </c>
-      <c r="AN3" s="48" t="s">
+      <c r="AM3" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="AN3" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="AO3" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="AP3" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="AO3" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="AP3" s="39" t="s">
+      <c r="AQ3" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="AQ3" s="38" t="s">
+      <c r="AR3" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="AR3" s="38" t="s">
+      <c r="AS3" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="AS3" s="38" t="s">
+      <c r="AT3" s="38" t="s">
         <v>134</v>
-      </c>
-      <c r="AT3" s="38" t="s">
-        <v>135</v>
       </c>
       <c r="AU3" s="38"/>
       <c r="AV3" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW3" s="38" t="n">
         <v>1</v>
       </c>
       <c r="AX3" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AY3" s="39" t="n">
         <v>45611</v>
@@ -2233,10 +2228,10 @@
         <v>45612</v>
       </c>
       <c r="BA3" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="BB3" s="38" t="s">
         <v>164</v>
-      </c>
-      <c r="BB3" s="38" t="s">
-        <v>165</v>
       </c>
       <c r="BC3" s="38"/>
       <c r="BD3" s="39"/>
@@ -2249,57 +2244,57 @@
       <c r="BK3" s="38"/>
       <c r="BL3" s="38"/>
       <c r="BM3" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN3" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BN3" s="38" t="s">
+      <c r="BO3" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP3" s="38" t="s">
         <v>141</v>
-      </c>
-      <c r="BO3" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="BP3" s="38" t="s">
-        <v>142</v>
       </c>
       <c r="BQ3" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="BR3" s="43" t="n">
+      <c r="BR3" s="42" t="n">
         <v>0.55</v>
       </c>
       <c r="BS3" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT3" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU3" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV3" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BT3" s="38" t="s">
+      <c r="BW3" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BX3" s="42" t="n">
+        <v>0.145833333333333</v>
+      </c>
+      <c r="BY3" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="BU3" s="38" t="s">
+      <c r="BZ3" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="BV3" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW3" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BX3" s="43" t="n">
-        <v>0.145833333333333</v>
-      </c>
-      <c r="BY3" s="38" t="s">
+      <c r="CA3" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="CB3" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="BZ3" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="CA3" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="CB3" s="38" t="s">
-        <v>144</v>
-      </c>
       <c r="CC3" s="39" t="n">
         <v>45612</v>
       </c>
-      <c r="CD3" s="43" t="n">
+      <c r="CD3" s="42" t="n">
         <v>0.28125</v>
       </c>
       <c r="CE3" s="39"/>
@@ -2310,23 +2305,29 @@
       <c r="CJ3" s="39"/>
       <c r="CK3" s="38"/>
       <c r="CL3" s="38"/>
-      <c r="CM3" s="42"/>
-      <c r="CN3" s="42"/>
+      <c r="CM3" s="41"/>
+      <c r="CN3" s="41"/>
       <c r="CO3" s="38"/>
       <c r="CP3" s="38"/>
-      <c r="CQ3" s="42"/>
-      <c r="CR3" s="42"/>
-      <c r="CS3" s="41"/>
+      <c r="CQ3" s="41"/>
+      <c r="CR3" s="41"/>
+      <c r="CS3" s="37"/>
       <c r="CT3" s="38"/>
       <c r="CU3" s="39"/>
       <c r="CV3" s="38"/>
+      <c r="CX3" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="CZ3" s="44" t="s">
+        <v>165</v>
+      </c>
     </row>
-    <row r="4" s="45" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="41" t="s">
+    <row r="4" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="37" t="s">
         <v>106</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>108</v>
@@ -2339,16 +2340,16 @@
         <v>45612</v>
       </c>
       <c r="G4" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="I4" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="I4" s="38" t="s">
-        <v>112</v>
-      </c>
       <c r="J4" s="38" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K4" s="40" t="s">
         <v>166</v>
@@ -2356,8 +2357,8 @@
       <c r="L4" s="40" t="s">
         <v>167</v>
       </c>
-      <c r="M4" s="41" t="s">
-        <v>115</v>
+      <c r="M4" s="37" t="s">
+        <v>114</v>
       </c>
       <c r="N4" s="40" t="s">
         <v>168</v>
@@ -2368,7 +2369,7 @@
       <c r="P4" s="38" t="s">
         <v>170</v>
       </c>
-      <c r="Q4" s="42" t="n">
+      <c r="Q4" s="41" t="n">
         <v>24306</v>
       </c>
       <c r="R4" s="40" t="s">
@@ -2378,10 +2379,10 @@
         <v>171</v>
       </c>
       <c r="T4" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="U4" s="38" t="s">
         <v>120</v>
-      </c>
-      <c r="U4" s="38" t="s">
-        <v>121</v>
       </c>
       <c r="V4" s="40" t="s">
         <v>172</v>
@@ -2419,48 +2420,48 @@
       <c r="AI4" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AJ4" s="43" t="s">
+      <c r="AJ4" s="42" t="s">
         <v>178</v>
       </c>
-      <c r="AK4" s="46" t="s">
+      <c r="AK4" s="45" t="s">
         <v>179</v>
       </c>
       <c r="AL4" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AM4" s="49" t="s">
+      <c r="AM4" s="48" t="s">
         <v>180</v>
       </c>
-      <c r="AN4" s="48" t="s">
+      <c r="AN4" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="AO4" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="AP4" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="AO4" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="AP4" s="39" t="s">
+      <c r="AQ4" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="AQ4" s="38" t="s">
+      <c r="AR4" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="AR4" s="38" t="s">
+      <c r="AS4" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="AS4" s="38" t="s">
+      <c r="AT4" s="38" t="s">
         <v>134</v>
-      </c>
-      <c r="AT4" s="38" t="s">
-        <v>135</v>
       </c>
       <c r="AU4" s="38"/>
       <c r="AV4" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW4" s="38" t="n">
         <v>1</v>
       </c>
       <c r="AX4" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AY4" s="39" t="n">
         <v>45611</v>
@@ -2469,10 +2470,10 @@
         <v>45612</v>
       </c>
       <c r="BA4" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="BB4" s="38" t="s">
         <v>164</v>
-      </c>
-      <c r="BB4" s="38" t="s">
-        <v>165</v>
       </c>
       <c r="BC4" s="38"/>
       <c r="BD4" s="39"/>
@@ -2485,57 +2486,57 @@
       <c r="BK4" s="38"/>
       <c r="BL4" s="38"/>
       <c r="BM4" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN4" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BN4" s="38" t="s">
+      <c r="BO4" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP4" s="38" t="s">
         <v>141</v>
-      </c>
-      <c r="BO4" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="BP4" s="38" t="s">
-        <v>142</v>
       </c>
       <c r="BQ4" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="BR4" s="43" t="n">
+      <c r="BR4" s="42" t="n">
         <v>0.972916666666667</v>
       </c>
       <c r="BS4" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT4" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU4" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV4" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BT4" s="38" t="s">
+      <c r="BW4" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BX4" s="42" t="n">
+        <v>0.145833333333333</v>
+      </c>
+      <c r="BY4" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="BU4" s="38" t="s">
+      <c r="BZ4" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="BV4" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW4" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BX4" s="43" t="n">
-        <v>0.145833333333333</v>
-      </c>
-      <c r="BY4" s="38" t="s">
+      <c r="CA4" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="CB4" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="BZ4" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="CA4" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="CB4" s="38" t="s">
-        <v>144</v>
-      </c>
       <c r="CC4" s="39" t="n">
         <v>45612</v>
       </c>
-      <c r="CD4" s="43" t="n">
+      <c r="CD4" s="42" t="n">
         <v>0.28125</v>
       </c>
       <c r="CE4" s="39"/>
@@ -2546,23 +2547,29 @@
       <c r="CJ4" s="39"/>
       <c r="CK4" s="38"/>
       <c r="CL4" s="38"/>
-      <c r="CM4" s="42"/>
-      <c r="CN4" s="42"/>
+      <c r="CM4" s="41"/>
+      <c r="CN4" s="41"/>
       <c r="CO4" s="38"/>
       <c r="CP4" s="38"/>
-      <c r="CQ4" s="42"/>
-      <c r="CR4" s="42"/>
-      <c r="CS4" s="41"/>
+      <c r="CQ4" s="41"/>
+      <c r="CR4" s="41"/>
+      <c r="CS4" s="37"/>
       <c r="CT4" s="38"/>
       <c r="CU4" s="39"/>
       <c r="CV4" s="38"/>
+      <c r="CX4" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="CZ4" s="44" t="s">
+        <v>165</v>
+      </c>
     </row>
-    <row r="5" s="45" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="41" t="s">
+    <row r="5" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="37" t="s">
         <v>106</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C5" s="38" t="s">
         <v>108</v>
@@ -2575,16 +2582,16 @@
         <v>45612</v>
       </c>
       <c r="G5" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="H5" s="38" t="s">
+      <c r="I5" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="I5" s="38" t="s">
-        <v>112</v>
-      </c>
       <c r="J5" s="38" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K5" s="40" t="s">
         <v>181</v>
@@ -2592,8 +2599,8 @@
       <c r="L5" s="40" t="s">
         <v>182</v>
       </c>
-      <c r="M5" s="41" t="s">
-        <v>150</v>
+      <c r="M5" s="37" t="s">
+        <v>149</v>
       </c>
       <c r="N5" s="40" t="s">
         <v>183</v>
@@ -2604,7 +2611,7 @@
       <c r="P5" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="Q5" s="42" t="n">
+      <c r="Q5" s="41" t="n">
         <v>28284</v>
       </c>
       <c r="R5" s="40" t="s">
@@ -2617,7 +2624,7 @@
         <v>187</v>
       </c>
       <c r="U5" s="38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="V5" s="40" t="s">
         <v>188</v>
@@ -2635,7 +2642,7 @@
         <v>45610</v>
       </c>
       <c r="AA5" s="39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="AB5" s="38" t="s">
         <v>191</v>
@@ -2661,48 +2668,48 @@
       <c r="AI5" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AJ5" s="43" t="n">
+      <c r="AJ5" s="42" t="n">
         <v>0.0416666666666667</v>
       </c>
-      <c r="AK5" s="46" t="s">
+      <c r="AK5" s="45" t="s">
         <v>195</v>
       </c>
       <c r="AL5" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AM5" s="49" t="s">
+      <c r="AM5" s="48" t="s">
         <v>196</v>
       </c>
-      <c r="AN5" s="48" t="s">
+      <c r="AN5" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="AO5" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="AP5" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="AO5" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="AP5" s="39" t="s">
+      <c r="AQ5" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="AQ5" s="38" t="s">
+      <c r="AR5" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="AR5" s="38" t="s">
+      <c r="AS5" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="AS5" s="38" t="s">
+      <c r="AT5" s="38" t="s">
         <v>134</v>
-      </c>
-      <c r="AT5" s="38" t="s">
-        <v>135</v>
       </c>
       <c r="AU5" s="38"/>
       <c r="AV5" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW5" s="38" t="n">
         <v>2</v>
       </c>
       <c r="AX5" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AY5" s="39" t="n">
         <v>45611</v>
@@ -2711,7 +2718,7 @@
         <v>45612</v>
       </c>
       <c r="BA5" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="BB5" s="38" t="s">
         <v>197</v>
@@ -2727,57 +2734,57 @@
       <c r="BK5" s="38"/>
       <c r="BL5" s="38"/>
       <c r="BM5" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN5" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BN5" s="38" t="s">
+      <c r="BO5" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP5" s="38" t="s">
         <v>141</v>
-      </c>
-      <c r="BO5" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="BP5" s="38" t="s">
-        <v>142</v>
       </c>
       <c r="BQ5" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="BR5" s="43" t="n">
+      <c r="BR5" s="42" t="n">
         <v>0.55</v>
       </c>
       <c r="BS5" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT5" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU5" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV5" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BT5" s="38" t="s">
+      <c r="BW5" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BX5" s="42" t="n">
+        <v>0.145833333333333</v>
+      </c>
+      <c r="BY5" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="BU5" s="38" t="s">
+      <c r="BZ5" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="BV5" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW5" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BX5" s="43" t="n">
-        <v>0.145833333333333</v>
-      </c>
-      <c r="BY5" s="38" t="s">
+      <c r="CA5" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="CB5" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="BZ5" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="CA5" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="CB5" s="38" t="s">
-        <v>144</v>
-      </c>
       <c r="CC5" s="39" t="n">
         <v>45612</v>
       </c>
-      <c r="CD5" s="43" t="n">
+      <c r="CD5" s="42" t="n">
         <v>0.28125</v>
       </c>
       <c r="CE5" s="39"/>
@@ -2788,23 +2795,29 @@
       <c r="CJ5" s="39"/>
       <c r="CK5" s="38"/>
       <c r="CL5" s="38"/>
-      <c r="CM5" s="42"/>
-      <c r="CN5" s="42"/>
+      <c r="CM5" s="41"/>
+      <c r="CN5" s="41"/>
       <c r="CO5" s="38"/>
       <c r="CP5" s="38"/>
-      <c r="CQ5" s="42"/>
-      <c r="CR5" s="42"/>
-      <c r="CS5" s="41"/>
+      <c r="CQ5" s="41"/>
+      <c r="CR5" s="41"/>
+      <c r="CS5" s="37"/>
       <c r="CT5" s="38"/>
       <c r="CU5" s="39"/>
       <c r="CV5" s="38"/>
+      <c r="CX5" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="CZ5" s="44" t="s">
+        <v>165</v>
+      </c>
     </row>
-    <row r="6" s="45" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="41" t="s">
+    <row r="6" s="44" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="37" t="s">
         <v>106</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>108</v>
@@ -2817,16 +2830,16 @@
         <v>45612</v>
       </c>
       <c r="G6" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="H6" s="38" t="s">
         <v>110</v>
       </c>
-      <c r="H6" s="38" t="s">
+      <c r="I6" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="I6" s="38" t="s">
-        <v>112</v>
-      </c>
       <c r="J6" s="38" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K6" s="40" t="s">
         <v>198</v>
@@ -2834,8 +2847,8 @@
       <c r="L6" s="40" t="s">
         <v>199</v>
       </c>
-      <c r="M6" s="41" t="s">
-        <v>150</v>
+      <c r="M6" s="37" t="s">
+        <v>149</v>
       </c>
       <c r="N6" s="40" t="s">
         <v>183</v>
@@ -2846,20 +2859,20 @@
       <c r="P6" s="38" t="s">
         <v>201</v>
       </c>
-      <c r="Q6" s="42" t="n">
+      <c r="Q6" s="41" t="n">
         <v>35966</v>
       </c>
       <c r="R6" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="S6" s="40" t="s">
+        <v>118</v>
+      </c>
+      <c r="T6" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="S6" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="T6" s="40" t="s">
+      <c r="U6" s="38" t="s">
         <v>120</v>
-      </c>
-      <c r="U6" s="38" t="s">
-        <v>121</v>
       </c>
       <c r="V6" s="40" t="s">
         <v>202</v>
@@ -2871,74 +2884,74 @@
         <v>203</v>
       </c>
       <c r="Y6" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="Z6" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="AA6" s="39" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB6" s="38" t="s">
         <v>124</v>
-      </c>
-      <c r="AB6" s="38" t="s">
-        <v>125</v>
       </c>
       <c r="AC6" s="39" t="n">
         <v>45610</v>
       </c>
       <c r="AD6" s="39" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AE6" s="38"/>
       <c r="AF6" s="38"/>
       <c r="AG6" s="38"/>
       <c r="AH6" s="40" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AI6" s="39" t="n">
         <v>45610</v>
       </c>
-      <c r="AJ6" s="43" t="s">
+      <c r="AJ6" s="42" t="s">
+        <v>126</v>
+      </c>
+      <c r="AK6" s="45" t="s">
         <v>127</v>
-      </c>
-      <c r="AK6" s="46" t="s">
-        <v>128</v>
       </c>
       <c r="AL6" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="AM6" s="49" t="s">
+      <c r="AM6" s="48" t="s">
         <v>204</v>
       </c>
-      <c r="AN6" s="48" t="s">
+      <c r="AN6" s="47" t="s">
+        <v>129</v>
+      </c>
+      <c r="AO6" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="AP6" s="39" t="s">
         <v>130</v>
       </c>
-      <c r="AO6" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="AP6" s="39" t="s">
+      <c r="AQ6" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="AQ6" s="38" t="s">
+      <c r="AR6" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="AR6" s="38" t="s">
+      <c r="AS6" s="38" t="s">
         <v>133</v>
       </c>
-      <c r="AS6" s="38" t="s">
+      <c r="AT6" s="38" t="s">
         <v>134</v>
-      </c>
-      <c r="AT6" s="38" t="s">
-        <v>135</v>
       </c>
       <c r="AU6" s="38"/>
       <c r="AV6" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AW6" s="38" t="n">
         <v>3</v>
       </c>
       <c r="AX6" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AY6" s="39" t="n">
         <v>45610</v>
@@ -2947,10 +2960,10 @@
         <v>45612</v>
       </c>
       <c r="BA6" s="38" t="s">
+        <v>137</v>
+      </c>
+      <c r="BB6" s="38" t="s">
         <v>138</v>
-      </c>
-      <c r="BB6" s="38" t="s">
-        <v>139</v>
       </c>
       <c r="BC6" s="38"/>
       <c r="BD6" s="39"/>
@@ -2963,57 +2976,57 @@
       <c r="BK6" s="38"/>
       <c r="BL6" s="38"/>
       <c r="BM6" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN6" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BN6" s="38" t="s">
+      <c r="BO6" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP6" s="38" t="s">
         <v>141</v>
-      </c>
-      <c r="BO6" s="38" t="s">
-        <v>140</v>
-      </c>
-      <c r="BP6" s="38" t="s">
-        <v>142</v>
       </c>
       <c r="BQ6" s="39" t="n">
         <v>45611</v>
       </c>
-      <c r="BR6" s="43" t="n">
+      <c r="BR6" s="42" t="n">
         <v>0.330555555555556</v>
       </c>
       <c r="BS6" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT6" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU6" s="38" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV6" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="BT6" s="38" t="s">
+      <c r="BW6" s="39" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BX6" s="42" t="n">
+        <v>0.145833333333333</v>
+      </c>
+      <c r="BY6" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="BU6" s="38" t="s">
+      <c r="BZ6" s="39" t="s">
         <v>140</v>
       </c>
-      <c r="BV6" s="38" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW6" s="39" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BX6" s="43" t="n">
-        <v>0.145833333333333</v>
-      </c>
-      <c r="BY6" s="38" t="s">
+      <c r="CA6" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="CB6" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="BZ6" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="CA6" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="CB6" s="38" t="s">
-        <v>144</v>
-      </c>
       <c r="CC6" s="39" t="n">
         <v>45612</v>
       </c>
-      <c r="CD6" s="43" t="n">
+      <c r="CD6" s="42" t="n">
         <v>0.28125</v>
       </c>
       <c r="CE6" s="39"/>
@@ -3024,34 +3037,40 @@
       <c r="CJ6" s="39"/>
       <c r="CK6" s="38"/>
       <c r="CL6" s="38" t="s">
-        <v>145</v>
-      </c>
-      <c r="CM6" s="42" t="n">
+        <v>144</v>
+      </c>
+      <c r="CM6" s="41" t="n">
         <v>42688</v>
       </c>
-      <c r="CN6" s="42" t="n">
+      <c r="CN6" s="41" t="n">
         <v>45611</v>
       </c>
       <c r="CO6" s="38"/>
       <c r="CP6" s="38" t="s">
-        <v>146</v>
-      </c>
-      <c r="CQ6" s="42" t="n">
+        <v>145</v>
+      </c>
+      <c r="CQ6" s="41" t="n">
         <v>45610</v>
       </c>
-      <c r="CR6" s="42" t="n">
+      <c r="CR6" s="41" t="n">
         <v>45611</v>
       </c>
-      <c r="CS6" s="41"/>
+      <c r="CS6" s="37"/>
       <c r="CT6" s="38"/>
       <c r="CU6" s="39"/>
       <c r="CV6" s="38"/>
+      <c r="CX6" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="CZ6" s="44" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E7" s="39"/>
       <c r="F7" s="39"/>
-      <c r="BR7" s="43"/>
-      <c r="BW7" s="50"/>
+      <c r="BR7" s="42"/>
+      <c r="BW7" s="49"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E8" s="39"/>
@@ -3110,29 +3129,29 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="10" width="14.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="3" width="14.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="3" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="51" width="15.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="50" width="15.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="10" width="15.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="10" width="17.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="29" min="29" style="5" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="52" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="53" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="30" min="30" style="51" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="31" min="31" style="52" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="32" style="10" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="34" min="33" style="10" width="11.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="35" style="10" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="51" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="50" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="10" width="7.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="54" width="8.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="54" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="53" width="8.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="53" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="10" width="6.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="10" width="11.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="10" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="54" width="8.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="54" width="9.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="53" width="8.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="53" width="9.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="10" width="7.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="10" width="12.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="10" width="8.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="54" width="8.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="54" width="9.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="53" width="8.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="50" min="50" style="53" width="9.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="51" style="10" width="7.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="10" width="12.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="1" width="7"/>
@@ -3161,12 +3180,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="76" min="76" style="6" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="77" min="77" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="78" min="78" style="10" width="13.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="79" style="54" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="80" min="80" style="54" width="10.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="79" min="79" style="53" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="80" min="80" style="53" width="10.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="81" min="81" style="10" width="9.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="82" min="82" style="10" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="83" min="83" style="54" width="11.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="84" min="84" style="54" width="11.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="83" min="83" style="53" width="11.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="84" min="84" style="53" width="11.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="85" min="85" style="10" width="10.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="86" min="86" style="10" width="14.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="87" min="87" style="10" width="11.85"/>
@@ -3190,13 +3209,13 @@
       <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="55" t="s">
+      <c r="D1" s="54" t="s">
         <v>205</v>
       </c>
-      <c r="E1" s="55" t="s">
+      <c r="E1" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="55" t="s">
+      <c r="F1" s="54" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="11" t="s">
@@ -3229,7 +3248,7 @@
       <c r="P1" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="56" t="s">
+      <c r="Q1" s="55" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="20" t="s">
@@ -3250,16 +3269,16 @@
       <c r="W1" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="X1" s="57" t="s">
+      <c r="X1" s="56" t="s">
         <v>41</v>
       </c>
       <c r="Y1" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="Z1" s="58" t="s">
+      <c r="Z1" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="AA1" s="59" t="s">
+      <c r="AA1" s="58" t="s">
         <v>38</v>
       </c>
       <c r="AB1" s="14" t="s">
@@ -3268,7 +3287,7 @@
       <c r="AC1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="AD1" s="60" t="s">
+      <c r="AD1" s="59" t="s">
         <v>35</v>
       </c>
       <c r="AE1" s="31" t="s">
@@ -3370,7 +3389,7 @@
       <c r="BK1" s="33" t="s">
         <v>74</v>
       </c>
-      <c r="BL1" s="61" t="s">
+      <c r="BL1" s="60" t="s">
         <v>75</v>
       </c>
       <c r="BM1" s="31" t="s">
@@ -3388,7 +3407,7 @@
       <c r="BQ1" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="BR1" s="61" t="s">
+      <c r="BR1" s="60" t="s">
         <v>81</v>
       </c>
       <c r="BS1" s="31" t="s">
@@ -3406,46 +3425,46 @@
       <c r="BW1" s="33" t="s">
         <v>86</v>
       </c>
-      <c r="BX1" s="61" t="s">
+      <c r="BX1" s="60" t="s">
         <v>87</v>
       </c>
       <c r="BY1" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="BZ1" s="62" t="s">
+      <c r="BZ1" s="61" t="s">
         <v>89</v>
       </c>
-      <c r="CA1" s="63" t="s">
+      <c r="CA1" s="62" t="s">
         <v>90</v>
       </c>
-      <c r="CB1" s="63" t="s">
+      <c r="CB1" s="62" t="s">
         <v>91</v>
       </c>
-      <c r="CC1" s="62" t="s">
+      <c r="CC1" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="CD1" s="62" t="s">
+      <c r="CD1" s="61" t="s">
         <v>93</v>
       </c>
-      <c r="CE1" s="63" t="s">
+      <c r="CE1" s="62" t="s">
         <v>94</v>
       </c>
-      <c r="CF1" s="63" t="s">
+      <c r="CF1" s="62" t="s">
         <v>95</v>
       </c>
-      <c r="CG1" s="62" t="s">
+      <c r="CG1" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="CH1" s="62" t="s">
+      <c r="CH1" s="61" t="s">
         <v>97</v>
       </c>
-      <c r="CI1" s="62" t="s">
+      <c r="CI1" s="61" t="s">
         <v>98</v>
       </c>
-      <c r="CJ1" s="62" t="s">
+      <c r="CJ1" s="61" t="s">
         <v>99</v>
       </c>
-      <c r="CK1" s="62" t="s">
+      <c r="CK1" s="61" t="s">
         <v>100</v>
       </c>
       <c r="CL1" s="34" t="s">
@@ -3468,23 +3487,23 @@
       <c r="A2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="64" t="s">
-        <v>147</v>
+      <c r="B2" s="63" t="s">
+        <v>146</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F2" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G2" s="41" t="s">
+      <c r="E2" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F2" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G2" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H2" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>106</v>
@@ -3492,37 +3511,37 @@
       <c r="J2" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K2" s="66" t="s">
+      <c r="K2" s="65" t="s">
         <v>208</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="M2" s="41" t="s">
-        <v>115</v>
-      </c>
-      <c r="N2" s="45" t="s">
+      <c r="M2" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="N2" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="O2" s="45" t="s">
+      <c r="O2" s="44" t="s">
         <v>211</v>
       </c>
-      <c r="P2" s="66" t="s">
+      <c r="P2" s="65" t="s">
         <v>212</v>
       </c>
-      <c r="Q2" s="65" t="n">
+      <c r="Q2" s="64" t="n">
         <v>34604</v>
       </c>
-      <c r="R2" s="45" t="s">
+      <c r="R2" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S2" s="45" t="s">
-        <v>120</v>
-      </c>
-      <c r="T2" s="45" t="s">
+      <c r="S2" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T2" s="44" t="s">
         <v>214</v>
       </c>
-      <c r="V2" s="45" t="s">
+      <c r="V2" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W2" s="9" t="n">
@@ -3531,44 +3550,44 @@
       <c r="X2" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y2" s="66"/>
+      <c r="Y2" s="65"/>
       <c r="Z2" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AA2" s="67" t="s">
+      <c r="AA2" s="66" t="s">
         <v>217</v>
       </c>
-      <c r="AB2" s="68" t="s">
+      <c r="AB2" s="67" t="s">
         <v>218</v>
       </c>
       <c r="AC2" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD2" s="69" t="n">
+      <c r="AD2" s="68" t="n">
         <v>0.548611111111111</v>
       </c>
       <c r="AE2" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF2" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF2" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG2" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH2" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH2" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI2" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ2" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK2" s="71" t="n">
+      <c r="AK2" s="70" t="n">
         <v>1</v>
       </c>
-      <c r="AL2" s="72" t="s">
+      <c r="AL2" s="71" t="s">
         <v>222</v>
       </c>
       <c r="AM2" s="9" t="n">
@@ -3578,13 +3597,13 @@
         <v>45614</v>
       </c>
       <c r="AO2" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AP2" s="10" t="s">
         <v>223</v>
       </c>
       <c r="AQ2" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR2" s="9" t="n">
         <v>45614</v>
@@ -3593,90 +3612,90 @@
         <v>45615</v>
       </c>
       <c r="AT2" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="AU2" s="10" t="s">
         <v>164</v>
-      </c>
-      <c r="AU2" s="10" t="s">
-        <v>165</v>
       </c>
       <c r="AW2" s="9"/>
       <c r="AX2" s="9"/>
-      <c r="BA2" s="72" t="s">
+      <c r="BA2" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB2" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB2" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC2" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD2" s="72" t="s">
+      <c r="BC2" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE2" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF2" s="74"/>
-      <c r="BG2" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH2" s="72" t="s">
+      <c r="BD2" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE2" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF2" s="73"/>
+      <c r="BG2" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI2" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ2" s="72" t="s">
+      <c r="BH2" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI2" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ2" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK2" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL2" s="75" t="n">
+      <c r="BL2" s="74" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM2" s="72" t="s">
+      <c r="BM2" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN2" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN2" s="73" t="s">
+      <c r="BO2" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP2" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO2" s="72" t="s">
+      <c r="BQ2" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR2" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS2" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT2" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU2" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV2" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP2" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ2" s="73" t="n">
-        <v>45614</v>
-      </c>
-      <c r="BR2" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS2" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT2" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU2" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV2" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW2" s="73" t="n">
+      <c r="BW2" s="72" t="n">
         <v>45615</v>
       </c>
-      <c r="BX2" s="74" t="n">
+      <c r="BX2" s="73" t="n">
         <v>0.0701388888888889</v>
       </c>
       <c r="BZ2" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="CA2" s="54" t="n">
-        <v>45612</v>
-      </c>
-      <c r="CB2" s="54" t="n">
+      <c r="CA2" s="53" t="n">
+        <v>45612</v>
+      </c>
+      <c r="CB2" s="53" t="n">
         <v>45613</v>
       </c>
       <c r="CC2" s="10" t="s">
@@ -3685,14 +3704,20 @@
       <c r="CD2" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="CE2" s="54" t="n">
-        <v>45612</v>
-      </c>
-      <c r="CF2" s="54" t="n">
+      <c r="CE2" s="53" t="n">
+        <v>45612</v>
+      </c>
+      <c r="CF2" s="53" t="n">
         <v>45613</v>
       </c>
       <c r="CG2" s="10" t="s">
         <v>225</v>
+      </c>
+      <c r="CL2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="CN2" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3700,22 +3725,22 @@
         <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E3" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F3" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G3" s="41" t="s">
+      <c r="E3" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F3" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G3" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>106</v>
@@ -3723,40 +3748,40 @@
       <c r="J3" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K3" s="66" t="s">
+      <c r="K3" s="65" t="s">
         <v>227</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="M3" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="N3" s="45" t="s">
+      <c r="M3" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="N3" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O3" s="45" t="s">
+      <c r="O3" s="44" t="s">
         <v>229</v>
       </c>
-      <c r="P3" s="66" t="s">
+      <c r="P3" s="65" t="s">
         <v>230</v>
       </c>
-      <c r="Q3" s="65" t="n">
+      <c r="Q3" s="64" t="n">
         <v>34938</v>
       </c>
-      <c r="R3" s="45" t="s">
+      <c r="R3" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S3" s="45" t="s">
+      <c r="S3" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T3" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U3" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T3" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U3" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V3" s="45" t="s">
+      <c r="V3" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W3" s="9" t="n">
@@ -3765,41 +3790,41 @@
       <c r="X3" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y3" s="66"/>
+      <c r="Y3" s="65"/>
       <c r="Z3" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AA3" s="67" t="s">
+      <c r="AA3" s="66" t="s">
         <v>232</v>
       </c>
-      <c r="AB3" s="68" t="s">
+      <c r="AB3" s="67" t="s">
         <v>233</v>
       </c>
       <c r="AC3" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD3" s="69" t="n">
+      <c r="AD3" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE3" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF3" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF3" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG3" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH3" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH3" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI3" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ3" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK3" s="71" t="n">
+      <c r="AK3" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL3" s="1" t="s">
@@ -3812,13 +3837,13 @@
         <v>45614</v>
       </c>
       <c r="AO3" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AP3" s="10" t="s">
         <v>234</v>
       </c>
       <c r="AQ3" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR3" s="9" t="n">
         <v>45614</v>
@@ -3827,103 +3852,109 @@
         <v>45615</v>
       </c>
       <c r="AT3" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AU3" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AW3" s="9"/>
       <c r="AX3" s="9"/>
-      <c r="BA3" s="72" t="s">
+      <c r="BA3" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB3" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB3" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC3" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD3" s="72" t="s">
+      <c r="BC3" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE3" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF3" s="74"/>
-      <c r="BG3" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH3" s="72" t="s">
+      <c r="BD3" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE3" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF3" s="73"/>
+      <c r="BG3" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI3" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ3" s="72" t="s">
+      <c r="BH3" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI3" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ3" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK3" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL3" s="75" t="n">
+      <c r="BL3" s="74" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM3" s="72" t="s">
+      <c r="BM3" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN3" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN3" s="73" t="s">
+      <c r="BO3" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP3" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO3" s="72" t="s">
+      <c r="BQ3" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR3" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS3" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT3" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU3" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV3" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP3" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ3" s="73" t="n">
+      <c r="BW3" s="72" t="n">
+        <v>45615</v>
+      </c>
+      <c r="BX3" s="73" t="n">
+        <v>0.0215277777777778</v>
+      </c>
+      <c r="BZ3" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="CA3" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="BR3" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS3" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT3" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU3" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV3" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW3" s="73" t="n">
-        <v>45615</v>
-      </c>
-      <c r="BX3" s="74" t="n">
-        <v>0.0215277777777778</v>
-      </c>
-      <c r="BZ3" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="CA3" s="54" t="n">
-        <v>45614</v>
-      </c>
-      <c r="CB3" s="54" t="n">
+      <c r="CB3" s="53" t="n">
         <v>45614</v>
       </c>
       <c r="CC3" s="10" t="s">
         <v>236</v>
       </c>
       <c r="CD3" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="CE3" s="54" t="n">
+        <v>145</v>
+      </c>
+      <c r="CE3" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="CF3" s="54" t="n">
+      <c r="CF3" s="53" t="n">
         <v>45615</v>
+      </c>
+      <c r="CL3" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="CN3" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3931,22 +3962,22 @@
         <v>106</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F4" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G4" s="41" t="s">
+      <c r="E4" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F4" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G4" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>106</v>
@@ -3954,40 +3985,40 @@
       <c r="J4" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K4" s="66" t="s">
+      <c r="K4" s="65" t="s">
         <v>237</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="M4" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="N4" s="45" t="s">
+      <c r="M4" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="N4" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O4" s="45" t="s">
+      <c r="O4" s="44" t="s">
         <v>200</v>
       </c>
-      <c r="P4" s="66" t="s">
+      <c r="P4" s="65" t="s">
         <v>239</v>
       </c>
-      <c r="Q4" s="65" t="n">
+      <c r="Q4" s="64" t="n">
         <v>34349</v>
       </c>
-      <c r="R4" s="45" t="s">
+      <c r="R4" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T4" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U4" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T4" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U4" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W4" s="9" t="n">
@@ -3996,43 +4027,43 @@
       <c r="X4" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y4" s="66" t="s">
+      <c r="Y4" s="65" t="s">
         <v>240</v>
       </c>
       <c r="Z4" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AA4" s="67" t="s">
+      <c r="AA4" s="66" t="s">
         <v>241</v>
       </c>
-      <c r="AB4" s="68" t="s">
+      <c r="AB4" s="67" t="s">
         <v>233</v>
       </c>
       <c r="AC4" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD4" s="69" t="n">
+      <c r="AD4" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE4" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF4" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF4" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG4" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH4" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH4" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI4" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ4" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK4" s="71" t="n">
+      <c r="AK4" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL4" s="1" t="s">
@@ -4045,13 +4076,13 @@
         <v>45614</v>
       </c>
       <c r="AO4" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AP4" s="10" t="s">
         <v>234</v>
       </c>
       <c r="AQ4" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR4" s="9" t="n">
         <v>45614</v>
@@ -4060,103 +4091,109 @@
         <v>45615</v>
       </c>
       <c r="AT4" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AU4" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AW4" s="9"/>
       <c r="AX4" s="9"/>
-      <c r="BA4" s="72" t="s">
+      <c r="BA4" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB4" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB4" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC4" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD4" s="72" t="s">
+      <c r="BC4" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE4" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF4" s="74"/>
-      <c r="BG4" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH4" s="72" t="s">
+      <c r="BD4" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE4" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF4" s="73"/>
+      <c r="BG4" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI4" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ4" s="72" t="s">
+      <c r="BH4" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI4" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ4" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK4" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL4" s="75" t="n">
+      <c r="BL4" s="74" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM4" s="72" t="s">
+      <c r="BM4" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN4" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN4" s="73" t="s">
+      <c r="BO4" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP4" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO4" s="72" t="s">
+      <c r="BQ4" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR4" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS4" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT4" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU4" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV4" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP4" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ4" s="73" t="n">
+      <c r="BW4" s="72" t="n">
+        <v>45615</v>
+      </c>
+      <c r="BX4" s="73" t="n">
+        <v>0.0701388888888889</v>
+      </c>
+      <c r="BZ4" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="CA4" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="BR4" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS4" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT4" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU4" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV4" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW4" s="73" t="n">
-        <v>45615</v>
-      </c>
-      <c r="BX4" s="74" t="n">
-        <v>0.0701388888888889</v>
-      </c>
-      <c r="BZ4" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="CA4" s="54" t="n">
-        <v>45614</v>
-      </c>
-      <c r="CB4" s="54" t="n">
+      <c r="CB4" s="53" t="n">
         <v>45614</v>
       </c>
       <c r="CC4" s="10" t="s">
         <v>236</v>
       </c>
       <c r="CD4" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="CE4" s="54" t="n">
+        <v>145</v>
+      </c>
+      <c r="CE4" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="CF4" s="54" t="n">
+      <c r="CF4" s="53" t="n">
         <v>45615</v>
+      </c>
+      <c r="CL4" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="CN4" s="1" t="s">
+        <v>165</v>
       </c>
       <c r="CO4" s="5"/>
     </row>
@@ -4165,22 +4202,22 @@
         <v>106</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E5" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F5" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G5" s="41" t="s">
+      <c r="E5" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F5" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G5" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>106</v>
@@ -4188,40 +4225,40 @@
       <c r="J5" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K5" s="66" t="s">
+      <c r="K5" s="65" t="s">
         <v>242</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>243</v>
       </c>
-      <c r="M5" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="N5" s="45" t="s">
+      <c r="M5" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="N5" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O5" s="45" t="s">
+      <c r="O5" s="44" t="s">
         <v>229</v>
       </c>
-      <c r="P5" s="66" t="s">
+      <c r="P5" s="65" t="s">
         <v>244</v>
       </c>
-      <c r="Q5" s="65" t="n">
+      <c r="Q5" s="64" t="n">
         <v>31324</v>
       </c>
-      <c r="R5" s="45" t="s">
+      <c r="R5" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S5" s="45" t="s">
+      <c r="S5" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T5" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U5" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T5" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U5" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V5" s="45" t="s">
+      <c r="V5" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W5" s="9" t="n">
@@ -4230,43 +4267,43 @@
       <c r="X5" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y5" s="66" t="s">
+      <c r="Y5" s="65" t="s">
         <v>245</v>
       </c>
       <c r="Z5" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AA5" s="67" t="s">
+      <c r="AA5" s="66" t="s">
         <v>241</v>
       </c>
-      <c r="AB5" s="68" t="s">
+      <c r="AB5" s="67" t="s">
         <v>233</v>
       </c>
       <c r="AC5" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD5" s="69" t="n">
+      <c r="AD5" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF5" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF5" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG5" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH5" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH5" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI5" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ5" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK5" s="71" t="n">
+      <c r="AK5" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL5" s="1" t="s">
@@ -4279,13 +4316,13 @@
         <v>45614</v>
       </c>
       <c r="AO5" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AP5" s="10" t="s">
         <v>234</v>
       </c>
       <c r="AQ5" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR5" s="9" t="n">
         <v>45614</v>
@@ -4294,103 +4331,109 @@
         <v>45615</v>
       </c>
       <c r="AT5" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AU5" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AW5" s="9"/>
       <c r="AX5" s="9"/>
-      <c r="BA5" s="72" t="s">
+      <c r="BA5" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB5" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB5" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC5" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD5" s="72" t="s">
+      <c r="BC5" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE5" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF5" s="74"/>
-      <c r="BG5" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH5" s="72" t="s">
+      <c r="BD5" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE5" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF5" s="73"/>
+      <c r="BG5" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI5" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ5" s="72" t="s">
+      <c r="BH5" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI5" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ5" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK5" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL5" s="75" t="n">
+      <c r="BL5" s="74" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM5" s="72" t="s">
+      <c r="BM5" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN5" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN5" s="73" t="s">
+      <c r="BO5" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP5" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO5" s="72" t="s">
+      <c r="BQ5" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR5" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS5" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT5" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU5" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV5" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP5" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ5" s="73" t="n">
+      <c r="BW5" s="72" t="n">
+        <v>45615</v>
+      </c>
+      <c r="BX5" s="73" t="n">
+        <v>0.0701388888888889</v>
+      </c>
+      <c r="BZ5" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="CA5" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="BR5" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS5" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT5" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU5" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV5" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW5" s="73" t="n">
-        <v>45615</v>
-      </c>
-      <c r="BX5" s="74" t="n">
-        <v>0.0701388888888889</v>
-      </c>
-      <c r="BZ5" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="CA5" s="54" t="n">
-        <v>45614</v>
-      </c>
-      <c r="CB5" s="54" t="n">
+      <c r="CB5" s="53" t="n">
         <v>45614</v>
       </c>
       <c r="CC5" s="10" t="s">
         <v>236</v>
       </c>
       <c r="CD5" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="CE5" s="54" t="n">
+        <v>145</v>
+      </c>
+      <c r="CE5" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="CF5" s="54" t="n">
+      <c r="CF5" s="53" t="n">
         <v>45615</v>
+      </c>
+      <c r="CL5" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="CN5" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4398,22 +4441,22 @@
         <v>106</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E6" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F6" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G6" s="41" t="s">
+      <c r="E6" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F6" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G6" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>106</v>
@@ -4421,40 +4464,40 @@
       <c r="J6" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K6" s="66" t="s">
+      <c r="K6" s="65" t="s">
         <v>246</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="M6" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="N6" s="45" t="s">
+      <c r="M6" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="N6" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O6" s="45" t="s">
+      <c r="O6" s="44" t="s">
         <v>229</v>
       </c>
-      <c r="P6" s="66" t="s">
+      <c r="P6" s="65" t="s">
         <v>248</v>
       </c>
-      <c r="Q6" s="65" t="n">
+      <c r="Q6" s="64" t="n">
         <v>34979</v>
       </c>
-      <c r="R6" s="45" t="s">
+      <c r="R6" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S6" s="45" t="s">
+      <c r="S6" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T6" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U6" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T6" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U6" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V6" s="45" t="s">
+      <c r="V6" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W6" s="9" t="n">
@@ -4463,43 +4506,43 @@
       <c r="X6" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y6" s="66" t="s">
+      <c r="Y6" s="65" t="s">
         <v>245</v>
       </c>
       <c r="Z6" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AA6" s="67" t="s">
+      <c r="AA6" s="66" t="s">
         <v>241</v>
       </c>
-      <c r="AB6" s="68" t="s">
+      <c r="AB6" s="67" t="s">
         <v>233</v>
       </c>
       <c r="AC6" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD6" s="69" t="n">
+      <c r="AD6" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE6" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF6" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF6" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG6" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH6" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH6" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI6" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ6" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK6" s="71" t="n">
+      <c r="AK6" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL6" s="1" t="s">
@@ -4512,13 +4555,13 @@
         <v>45614</v>
       </c>
       <c r="AO6" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AP6" s="10" t="s">
         <v>234</v>
       </c>
       <c r="AQ6" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR6" s="9" t="n">
         <v>45614</v>
@@ -4527,103 +4570,109 @@
         <v>45615</v>
       </c>
       <c r="AT6" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AU6" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AW6" s="9"/>
       <c r="AX6" s="9"/>
-      <c r="BA6" s="72" t="s">
+      <c r="BA6" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB6" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB6" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC6" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD6" s="72" t="s">
+      <c r="BC6" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE6" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF6" s="74"/>
-      <c r="BG6" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH6" s="72" t="s">
+      <c r="BD6" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE6" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF6" s="73"/>
+      <c r="BG6" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI6" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ6" s="72" t="s">
+      <c r="BH6" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI6" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ6" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK6" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL6" s="75" t="n">
+      <c r="BL6" s="74" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM6" s="72" t="s">
+      <c r="BM6" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN6" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN6" s="73" t="s">
+      <c r="BO6" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP6" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO6" s="72" t="s">
+      <c r="BQ6" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR6" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS6" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT6" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU6" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV6" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP6" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ6" s="73" t="n">
+      <c r="BW6" s="72" t="n">
+        <v>45615</v>
+      </c>
+      <c r="BX6" s="73" t="n">
+        <v>0.0701388888888889</v>
+      </c>
+      <c r="BZ6" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="CA6" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="BR6" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS6" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT6" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU6" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV6" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW6" s="73" t="n">
-        <v>45615</v>
-      </c>
-      <c r="BX6" s="74" t="n">
-        <v>0.0701388888888889</v>
-      </c>
-      <c r="BZ6" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="CA6" s="54" t="n">
-        <v>45614</v>
-      </c>
-      <c r="CB6" s="54" t="n">
+      <c r="CB6" s="53" t="n">
         <v>45614</v>
       </c>
       <c r="CC6" s="10" t="s">
         <v>236</v>
       </c>
       <c r="CD6" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="CE6" s="54" t="n">
+        <v>145</v>
+      </c>
+      <c r="CE6" s="53" t="n">
         <v>45614</v>
       </c>
-      <c r="CF6" s="54" t="n">
+      <c r="CF6" s="53" t="n">
         <v>45615</v>
+      </c>
+      <c r="CL6" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="CN6" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4631,22 +4680,22 @@
         <v>106</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E7" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F7" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G7" s="41" t="s">
+      <c r="E7" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F7" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G7" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>106</v>
@@ -4654,40 +4703,40 @@
       <c r="J7" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K7" s="66" t="s">
+      <c r="K7" s="65" t="s">
         <v>249</v>
       </c>
       <c r="L7" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="M7" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="N7" s="45" t="s">
+      <c r="M7" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="N7" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O7" s="45" t="s">
+      <c r="O7" s="44" t="s">
         <v>251</v>
       </c>
-      <c r="P7" s="66" t="s">
+      <c r="P7" s="65" t="s">
         <v>252</v>
       </c>
-      <c r="Q7" s="65" t="n">
+      <c r="Q7" s="64" t="n">
         <v>37351</v>
       </c>
-      <c r="R7" s="45" t="s">
+      <c r="R7" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S7" s="45" t="s">
+      <c r="S7" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T7" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U7" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T7" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U7" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V7" s="45" t="s">
+      <c r="V7" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W7" s="9" t="n">
@@ -4696,43 +4745,43 @@
       <c r="X7" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="Y7" s="66" t="s">
+      <c r="Y7" s="65" t="s">
         <v>245</v>
       </c>
       <c r="Z7" s="9" t="n">
         <v>45616</v>
       </c>
-      <c r="AA7" s="67" t="s">
+      <c r="AA7" s="66" t="s">
         <v>254</v>
       </c>
-      <c r="AB7" s="68" t="s">
+      <c r="AB7" s="67" t="s">
         <v>233</v>
       </c>
       <c r="AC7" s="9" t="n">
         <v>45616</v>
       </c>
-      <c r="AD7" s="69" t="n">
+      <c r="AD7" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE7" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF7" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF7" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG7" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH7" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH7" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI7" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ7" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK7" s="71" t="n">
+      <c r="AK7" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL7" s="1" t="s">
@@ -4745,13 +4794,13 @@
         <v>45615</v>
       </c>
       <c r="AO7" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AP7" s="10" t="s">
         <v>255</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR7" s="9" t="n">
         <v>45615</v>
@@ -4760,94 +4809,100 @@
         <v>45616</v>
       </c>
       <c r="AT7" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AU7" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AW7" s="9"/>
       <c r="AX7" s="9"/>
-      <c r="BA7" s="72" t="s">
+      <c r="BA7" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB7" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB7" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC7" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD7" s="72" t="s">
+      <c r="BC7" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE7" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF7" s="74"/>
-      <c r="BG7" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH7" s="72" t="s">
+      <c r="BD7" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE7" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF7" s="73"/>
+      <c r="BG7" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI7" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ7" s="72" t="s">
+      <c r="BH7" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI7" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ7" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK7" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="BL7" s="75" t="n">
+      <c r="BL7" s="74" t="n">
         <v>0.59375</v>
       </c>
-      <c r="BM7" s="72" t="s">
+      <c r="BM7" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN7" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN7" s="73" t="s">
+      <c r="BO7" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP7" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO7" s="72" t="s">
+      <c r="BQ7" s="72" t="n">
+        <v>45615</v>
+      </c>
+      <c r="BR7" s="74" t="n">
+        <v>0.6875</v>
+      </c>
+      <c r="BS7" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT7" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU7" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV7" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP7" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ7" s="73" t="n">
+      <c r="BW7" s="72" t="n">
+        <v>45616</v>
+      </c>
+      <c r="BX7" s="73" t="n">
+        <v>0.0472222222222222</v>
+      </c>
+      <c r="BZ7" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="CA7" s="53" t="n">
         <v>45615</v>
       </c>
-      <c r="BR7" s="75" t="n">
-        <v>0.6875</v>
-      </c>
-      <c r="BS7" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT7" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU7" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV7" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW7" s="73" t="n">
-        <v>45616</v>
-      </c>
-      <c r="BX7" s="74" t="n">
-        <v>0.0472222222222222</v>
-      </c>
-      <c r="BZ7" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="CA7" s="54" t="n">
-        <v>45615</v>
-      </c>
-      <c r="CB7" s="54" t="n">
+      <c r="CB7" s="53" t="n">
         <v>45616</v>
       </c>
       <c r="CC7" s="10" t="s">
         <v>236</v>
+      </c>
+      <c r="CL7" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="CN7" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4855,22 +4910,22 @@
         <v>106</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E8" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F8" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G8" s="41" t="s">
+      <c r="E8" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F8" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G8" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>106</v>
@@ -4878,40 +4933,40 @@
       <c r="J8" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K8" s="66" t="s">
+      <c r="K8" s="65" t="s">
         <v>256</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="M8" s="41" t="s">
-        <v>150</v>
-      </c>
-      <c r="N8" s="45" t="s">
+      <c r="M8" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="N8" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O8" s="45" t="s">
+      <c r="O8" s="44" t="s">
         <v>258</v>
       </c>
-      <c r="P8" s="66" t="s">
+      <c r="P8" s="65" t="s">
         <v>259</v>
       </c>
-      <c r="Q8" s="65" t="n">
+      <c r="Q8" s="64" t="n">
         <v>30591</v>
       </c>
-      <c r="R8" s="45" t="s">
+      <c r="R8" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S8" s="45" t="s">
+      <c r="S8" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T8" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U8" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T8" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U8" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V8" s="45" t="s">
+      <c r="V8" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W8" s="9" t="n">
@@ -4920,7 +4975,7 @@
       <c r="X8" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y8" s="66" t="s">
+      <c r="Y8" s="65" t="s">
         <v>260</v>
       </c>
       <c r="Z8" s="9" t="n">
@@ -4929,34 +4984,34 @@
       <c r="AA8" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="AB8" s="45" t="s">
+      <c r="AB8" s="44" t="s">
         <v>233</v>
       </c>
       <c r="AC8" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD8" s="69" t="n">
+      <c r="AD8" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE8" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF8" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF8" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG8" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH8" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH8" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI8" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ8" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK8" s="71" t="n">
+      <c r="AK8" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL8" s="10" t="s">
@@ -4969,13 +5024,13 @@
         <v>45614</v>
       </c>
       <c r="AO8" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AP8" s="10" t="s">
         <v>223</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR8" s="9" t="n">
         <v>45614</v>
@@ -4984,90 +5039,90 @@
         <v>45615</v>
       </c>
       <c r="AT8" s="10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AU8" s="10" t="s">
         <v>261</v>
       </c>
       <c r="AW8" s="9"/>
       <c r="AX8" s="9"/>
-      <c r="BA8" s="72" t="s">
+      <c r="BA8" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB8" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB8" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC8" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD8" s="72" t="s">
+      <c r="BC8" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE8" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF8" s="74"/>
-      <c r="BG8" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BH8" s="72" t="s">
+      <c r="BD8" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE8" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF8" s="73"/>
+      <c r="BG8" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BI8" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BJ8" s="72" t="s">
+      <c r="BH8" s="71" t="s">
         <v>141</v>
+      </c>
+      <c r="BI8" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BJ8" s="71" t="s">
+        <v>140</v>
       </c>
       <c r="BK8" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL8" s="75" t="n">
+      <c r="BL8" s="74" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM8" s="72" t="s">
+      <c r="BM8" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN8" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN8" s="73" t="s">
+      <c r="BO8" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP8" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO8" s="72" t="s">
+      <c r="BQ8" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR8" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS8" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT8" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU8" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV8" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP8" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ8" s="73" t="n">
-        <v>45614</v>
-      </c>
-      <c r="BR8" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS8" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT8" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU8" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV8" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW8" s="73" t="n">
+      <c r="BW8" s="72" t="n">
         <v>45615</v>
       </c>
-      <c r="BX8" s="74" t="n">
+      <c r="BX8" s="73" t="n">
         <v>0.0215277777777778</v>
       </c>
       <c r="BZ8" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="CA8" s="54" t="n">
-        <v>45612</v>
-      </c>
-      <c r="CB8" s="54" t="n">
+      <c r="CA8" s="53" t="n">
+        <v>45612</v>
+      </c>
+      <c r="CB8" s="53" t="n">
         <v>45613</v>
       </c>
       <c r="CC8" s="10" t="s">
@@ -5076,14 +5131,20 @@
       <c r="CD8" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="CE8" s="54" t="n">
-        <v>45612</v>
-      </c>
-      <c r="CF8" s="54" t="n">
+      <c r="CE8" s="53" t="n">
+        <v>45612</v>
+      </c>
+      <c r="CF8" s="53" t="n">
         <v>45613</v>
       </c>
       <c r="CG8" s="10" t="s">
         <v>225</v>
+      </c>
+      <c r="CL8" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="CN8" s="1" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5091,22 +5152,22 @@
         <v>106</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E9" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="F9" s="65" t="n">
-        <v>45612</v>
-      </c>
-      <c r="G9" s="41" t="s">
+      <c r="E9" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="F9" s="64" t="n">
+        <v>45612</v>
+      </c>
+      <c r="G9" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>106</v>
@@ -5114,40 +5175,40 @@
       <c r="J9" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="K9" s="66" t="s">
+      <c r="K9" s="65" t="s">
         <v>262</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="M9" s="41" t="s">
-        <v>115</v>
-      </c>
-      <c r="N9" s="45" t="s">
+      <c r="M9" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="N9" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="O9" s="45" t="s">
+      <c r="O9" s="44" t="s">
         <v>229</v>
       </c>
-      <c r="P9" s="66" t="s">
+      <c r="P9" s="65" t="s">
         <v>264</v>
       </c>
-      <c r="Q9" s="65" t="n">
+      <c r="Q9" s="64" t="n">
         <v>36207</v>
       </c>
-      <c r="R9" s="45" t="s">
+      <c r="R9" s="44" t="s">
         <v>213</v>
       </c>
-      <c r="S9" s="45" t="s">
+      <c r="S9" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="T9" s="44" t="s">
+        <v>231</v>
+      </c>
+      <c r="U9" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="T9" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="U9" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="V9" s="45" t="s">
+      <c r="V9" s="44" t="s">
         <v>215</v>
       </c>
       <c r="W9" s="9" t="n">
@@ -5156,7 +5217,7 @@
       <c r="X9" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="Y9" s="66" t="s">
+      <c r="Y9" s="65" t="s">
         <v>240</v>
       </c>
       <c r="Z9" s="9" t="n">
@@ -5165,34 +5226,34 @@
       <c r="AA9" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="AB9" s="45" t="s">
+      <c r="AB9" s="44" t="s">
         <v>233</v>
       </c>
       <c r="AC9" s="9" t="n">
         <v>45615</v>
       </c>
-      <c r="AD9" s="69" t="n">
+      <c r="AD9" s="68" t="n">
         <v>0.527777777777778</v>
       </c>
       <c r="AE9" s="38" t="s">
-        <v>132</v>
-      </c>
-      <c r="AF9" s="70" t="s">
+        <v>131</v>
+      </c>
+      <c r="AF9" s="69" t="s">
         <v>219</v>
       </c>
       <c r="AG9" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="AH9" s="70" t="s">
+        <v>133</v>
+      </c>
+      <c r="AH9" s="69" t="s">
         <v>220</v>
       </c>
       <c r="AI9" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="AJ9" s="10" t="s">
         <v>221</v>
       </c>
-      <c r="AK9" s="71" t="n">
+      <c r="AK9" s="70" t="n">
         <v>3</v>
       </c>
       <c r="AL9" s="10" t="s">
@@ -5205,13 +5266,13 @@
         <v>45614</v>
       </c>
       <c r="AO9" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AP9" s="10" t="s">
         <v>223</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AR9" s="9" t="n">
         <v>45614</v>
@@ -5220,40 +5281,40 @@
         <v>45615</v>
       </c>
       <c r="AT9" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AU9" s="10" t="s">
         <v>235</v>
       </c>
       <c r="AW9" s="9"/>
       <c r="AX9" s="9"/>
-      <c r="BA9" s="72" t="s">
+      <c r="BA9" s="71" t="s">
+        <v>142</v>
+      </c>
+      <c r="BB9" s="71" t="s">
         <v>143</v>
       </c>
-      <c r="BB9" s="72" t="s">
-        <v>144</v>
-      </c>
-      <c r="BC9" s="72" t="s">
-        <v>143</v>
-      </c>
-      <c r="BD9" s="72" t="s">
+      <c r="BC9" s="71" t="s">
         <v>142</v>
       </c>
-      <c r="BE9" s="73" t="n">
-        <v>45612</v>
-      </c>
-      <c r="BF9" s="74"/>
+      <c r="BD9" s="71" t="s">
+        <v>141</v>
+      </c>
+      <c r="BE9" s="72" t="n">
+        <v>45612</v>
+      </c>
+      <c r="BF9" s="73"/>
       <c r="BG9" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="BH9" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="BI9" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="BI9" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="BJ9" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="BK9" s="9" t="n">
         <v>45614</v>
@@ -5261,49 +5322,49 @@
       <c r="BL9" s="6" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="BM9" s="72" t="s">
+      <c r="BM9" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BN9" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BN9" s="73" t="s">
+      <c r="BO9" s="71" t="s">
+        <v>139</v>
+      </c>
+      <c r="BP9" s="71" t="s">
         <v>141</v>
       </c>
-      <c r="BO9" s="72" t="s">
+      <c r="BQ9" s="72" t="n">
+        <v>45614</v>
+      </c>
+      <c r="BR9" s="74" t="n">
+        <v>0.506944444444444</v>
+      </c>
+      <c r="BS9" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BT9" s="72" t="s">
+        <v>141</v>
+      </c>
+      <c r="BU9" s="72" t="s">
+        <v>139</v>
+      </c>
+      <c r="BV9" s="72" t="s">
         <v>140</v>
       </c>
-      <c r="BP9" s="72" t="s">
-        <v>142</v>
-      </c>
-      <c r="BQ9" s="73" t="n">
-        <v>45614</v>
-      </c>
-      <c r="BR9" s="75" t="n">
-        <v>0.506944444444444</v>
-      </c>
-      <c r="BS9" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BT9" s="73" t="s">
-        <v>142</v>
-      </c>
-      <c r="BU9" s="73" t="s">
-        <v>140</v>
-      </c>
-      <c r="BV9" s="73" t="s">
-        <v>141</v>
-      </c>
-      <c r="BW9" s="73" t="n">
+      <c r="BW9" s="72" t="n">
         <v>45615</v>
       </c>
-      <c r="BX9" s="74" t="n">
+      <c r="BX9" s="73" t="n">
         <v>0.0284722222222222</v>
       </c>
       <c r="BZ9" s="10" t="s">
         <v>224</v>
       </c>
-      <c r="CA9" s="54" t="n">
-        <v>45612</v>
-      </c>
-      <c r="CB9" s="54" t="n">
+      <c r="CA9" s="53" t="n">
+        <v>45612</v>
+      </c>
+      <c r="CB9" s="53" t="n">
         <v>45613</v>
       </c>
       <c r="CC9" s="10" t="s">
@@ -5312,14 +5373,20 @@
       <c r="CD9" s="10" t="s">
         <v>226</v>
       </c>
-      <c r="CE9" s="54" t="n">
-        <v>45612</v>
-      </c>
-      <c r="CF9" s="54" t="n">
+      <c r="CE9" s="53" t="n">
+        <v>45612</v>
+      </c>
+      <c r="CF9" s="53" t="n">
         <v>45613</v>
       </c>
       <c r="CG9" s="10" t="s">
         <v>225</v>
+      </c>
+      <c r="CL9" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="CN9" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>